<commit_message>
[IMP] assets_management: new test
</commit_message>
<xml_diff>
--- a/assets_management/tests/Test Workflow.xlsx
+++ b/assets_management/tests/Test Workflow.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="124">
   <si>
     <t xml:space="preserve">English</t>
   </si>
@@ -237,16 +237,10 @@
     <t xml:space="preserve">Valore bene</t>
   </si>
   <si>
-    <t xml:space="preserve"># giorni 2020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QA 2020</t>
-  </si>
-  <si>
-    <t xml:space="preserve"># giorni 2021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QA 2021</t>
+    <t xml:space="preserve"># giorni anno-1 (pre svalutazione)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QA anno-1 (pre svalutazione)</t>
   </si>
   <si>
     <t xml:space="preserve">Quota 90 giorni</t>
@@ -258,10 +252,10 @@
     <t xml:space="preserve">Q.A. dopo svalutaz,</t>
   </si>
   <si>
-    <t xml:space="preserve"># giorni residui 2021</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QA 2021 residua</t>
+    <t xml:space="preserve"># giorni anno-1 (post svalutazione)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QA anno-1 (post svalutazione)</t>
   </si>
   <si>
     <t xml:space="preserve">Quota 275 giorni</t>
@@ -294,46 +288,115 @@
     <t xml:space="preserve">asset_1.purchase_amount</t>
   </si>
   <si>
-    <t xml:space="preserve">asset_1.depreciation_amount[1]</t>
+    <t xml:space="preserve">asset_1.depreciation_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_1.depreciated_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_1.residual_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_1.depreciation_amount[-1]</t>
   </si>
   <si>
     <t xml:space="preserve">asset_1.depreciated_amount[-1]</t>
   </si>
   <si>
+    <t xml:space="preserve">asset_1.residual_amount[-1]</t>
+  </si>
+  <si>
     <t xml:space="preserve">asset_2.initial_amount</t>
   </si>
   <si>
     <t xml:space="preserve">asset_2.purchase_amount</t>
   </si>
   <si>
-    <t xml:space="preserve">asset_2.depreciation_amount[1]</t>
+    <t xml:space="preserve">asset_2.depreciation_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_2.depreciated_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_2.residual_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_2.depreciation_amount[-1]</t>
   </si>
   <si>
     <t xml:space="preserve">asset_2.depreciated_amount[-1]</t>
   </si>
   <si>
+    <t xml:space="preserve">asset_2.residual_amount[-1]</t>
+  </si>
+  <si>
     <t xml:space="preserve">asset_3.initial_amount</t>
   </si>
   <si>
     <t xml:space="preserve">asset_3.purchase_amount</t>
   </si>
   <si>
-    <t xml:space="preserve">asset_3.depreciation_amount[1]</t>
+    <t xml:space="preserve">asset_3.depreciation_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_3.depreciated_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_3.residual_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_3.depreciation_amount_pre[-1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_3.depreciated_amount_pre[-1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_3.residual_amount_pre[-1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_3.down_value[-1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_3.depreciation_amount_post[-1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_3.purchase_amount_post[-1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_3.residual_amount[_post[-1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_3.depreciation_amount[-1]</t>
   </si>
   <si>
     <t xml:space="preserve">asset_3.depreciated_amount[-1]</t>
   </si>
   <si>
+    <t xml:space="preserve">asset_3.residual_amount[-1]</t>
+  </si>
+  <si>
     <t xml:space="preserve">asset_4.initial_amount</t>
   </si>
   <si>
     <t xml:space="preserve">asset_4.purchase_amount</t>
   </si>
   <si>
-    <t xml:space="preserve">asset_4.depreciation_amount[1]</t>
+    <t xml:space="preserve">asset_4.depreciation_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_4.depreciated_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_4.residual_amount[-2]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_4.depreciation_amount[-1]</t>
   </si>
   <si>
     <t xml:space="preserve">asset_4.depreciated_amount[-1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asset_4.residual_amount[-1]</t>
   </si>
 </sst>
 </file>
@@ -627,11 +690,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -823,8 +886,8 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="91.56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="99.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="6.39"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="14.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="6.39"/>
   </cols>
   <sheetData>
     <row r="1" s="3" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -865,7 +928,7 @@
       <c r="M3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="N3" s="0" t="n">
+      <c r="N3" s="1" t="n">
         <v>365</v>
       </c>
     </row>
@@ -2575,7 +2638,7 @@
   <dimension ref="A1:AMJ37"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="28.93"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="10.39"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.72"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="47.56"/>
@@ -2629,7 +2692,7 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>70</v>
+        <v>29</v>
       </c>
       <c r="B3" s="12" t="n">
         <v>183</v>
@@ -2647,7 +2710,7 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>71</v>
+        <v>32</v>
       </c>
       <c r="B4" s="9" t="n">
         <f aca="false">G3/2</f>
@@ -2670,7 +2733,7 @@
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B5" s="12" t="n">
         <v>90</v>
@@ -2681,7 +2744,7 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">$G$3*B5/365</f>
@@ -2693,12 +2756,12 @@
       </c>
       <c r="D6" s="10"/>
       <c r="E6" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B7" s="8" t="n">
         <v>725</v>
@@ -2712,7 +2775,7 @@
         <v>275</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="G7" s="10" t="n">
         <f aca="false">D7*G2</f>
@@ -2721,7 +2784,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B8" s="28" t="n">
         <f aca="false">365-B5</f>
@@ -2732,7 +2795,7 @@
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B9" s="9" t="n">
         <f aca="false">$G$7*B8/365</f>
@@ -2744,12 +2807,12 @@
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B10" s="12" t="n">
         <v>31</v>
@@ -2760,7 +2823,7 @@
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">$G$7*B10/365</f>
@@ -3018,7 +3081,7 @@
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>53</v>
@@ -3058,7 +3121,7 @@
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B31" s="29" t="n">
         <f aca="false">B7</f>
@@ -3107,7 +3170,7 @@
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>53</v>
@@ -3288,7 +3351,7 @@
       </c>
       <c r="D4" s="10"/>
       <c r="E4" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>34</v>
@@ -3343,7 +3406,7 @@
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">C7*$G$4</f>
@@ -3990,24 +4053,24 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B45"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="27.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32.41"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="30" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="30" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="B1" s="30" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>88</v>
       </c>
       <c r="B2" s="31" t="n">
         <f aca="false">'Completo #1'!$B$2</f>
@@ -4015,8 +4078,8 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>89</v>
+      <c r="A3" s="1" t="s">
+        <v>87</v>
       </c>
       <c r="B3" s="31" t="n">
         <f aca="false">'Completo #1'!$B$4</f>
@@ -4024,117 +4087,324 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>90</v>
+      <c r="A4" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="B4" s="31" t="n">
         <f aca="false">B3</f>
         <v>125</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" s="31" t="n">
+        <f aca="false">'Completo #1'!$C$4</f>
+        <v>875</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6" s="31" t="n">
+        <f aca="false">'Completo #1'!$B$5</f>
+        <v>250</v>
+      </c>
+    </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B7" s="30" t="n">
+      <c r="B7" s="31" t="n">
+        <f aca="false">B4+B6</f>
+        <v>375</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B8" s="31" t="n">
+        <f aca="false">'Completo #1'!$C$5</f>
+        <v>625</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" s="30" t="n">
         <v>250</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>92</v>
-      </c>
-      <c r="B8" s="31" t="n">
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" s="31" t="n">
         <f aca="false">'Completo #2'!$B$2</f>
         <v>2500</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>93</v>
-      </c>
-      <c r="B9" s="31" t="n">
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="B13" s="31" t="n">
         <f aca="false">'Completo #2'!$B$4</f>
         <v>151.232876712329</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>94</v>
-      </c>
-      <c r="B10" s="31" t="n">
-        <f aca="false">B9</f>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="31" t="n">
+        <f aca="false">B13</f>
         <v>151.232876712329</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="B13" s="30" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>96</v>
-      </c>
-      <c r="B14" s="31" t="n">
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B15" s="31" t="n">
+        <f aca="false">'Completo #2'!$C$4</f>
+        <v>2348.76712328767</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="31" t="n">
+        <f aca="false">'Completo #2'!$B$5</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" s="31" t="n">
+        <f aca="false">B14+B16</f>
+        <v>751.232876712329</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B18" s="31" t="n">
+        <f aca="false">'Completo #2'!$C$5</f>
+        <v>1748.76712328767</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B21" s="30" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B22" s="31" t="n">
         <f aca="false">'Svalutazione #3'!$B$2</f>
         <v>1000</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>97</v>
-      </c>
-      <c r="B15" s="31" t="n">
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" s="31" t="n">
         <f aca="false">'Svalutazione #3'!$B$4</f>
         <v>125</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>98</v>
-      </c>
-      <c r="B16" s="31" t="n">
-        <f aca="false">B15</f>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B24" s="31" t="n">
+        <f aca="false">B23</f>
         <v>125</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
-        <v>99</v>
-      </c>
-      <c r="B19" s="30" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
-        <v>100</v>
-      </c>
-      <c r="B20" s="31" t="n">
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B25" s="31" t="n">
+        <f aca="false">'Svalutazione #3'!$C$4</f>
+        <v>875</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B26" s="31" t="n">
+        <f aca="false">'Svalutazione #3'!$B$6</f>
+        <v>61.6438356164384</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B27" s="31" t="n">
+        <f aca="false">B24+B26</f>
+        <v>186.643835616438</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B28" s="31" t="n">
+        <f aca="false">'Svalutazione #3'!$C$6</f>
+        <v>813.356164383562</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B29" s="31" t="n">
+        <f aca="false">'Svalutazione #3'!$B$7</f>
+        <v>725</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B30" s="31" t="n">
+        <f aca="false">'Svalutazione #3'!B9</f>
+        <v>51.7979452054795</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B31" s="31" t="n">
+        <f aca="false">'Svalutazione #3'!D7</f>
+        <v>275</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B32" s="31" t="n">
+        <f aca="false">'Svalutazione #3'!$C$9</f>
+        <v>36.5582191780822</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B33" s="31" t="n">
+        <f aca="false">B26+B30</f>
+        <v>113.441780821918</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="B34" s="31" t="n">
+        <f aca="false">B23+B26+B30</f>
+        <v>238.441780821918</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="B35" s="31" t="n">
+        <f aca="false">'Svalutazione #3'!$C$9</f>
+        <v>36.5582191780822</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="B38" s="30" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B39" s="31" t="n">
         <f aca="false">'Parziale #4'!$B$2</f>
         <v>2500</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
-        <v>101</v>
-      </c>
-      <c r="B21" s="31" t="n">
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="B40" s="31" t="n">
         <f aca="false">'Parziale #4'!$B$4</f>
         <v>151.232876712329</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
-        <v>102</v>
-      </c>
-      <c r="B22" s="31" t="n">
-        <f aca="false">B21</f>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="B41" s="31" t="n">
+        <f aca="false">B40</f>
         <v>151.232876712329</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B42" s="31" t="n">
+        <f aca="false">'Parziale #4'!$C$4</f>
+        <v>2348.76712328767</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B43" s="31" t="n">
+        <f aca="false">'Parziale #4'!$B$5</f>
+        <v>600</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B44" s="31" t="n">
+        <f aca="false">B41+B43</f>
+        <v>751.232876712329</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B45" s="31" t="n">
+        <f aca="false">'Parziale #4'!$C$5</f>
+        <v>1748.76712328767</v>
       </c>
     </row>
   </sheetData>

</xml_diff>